<commit_message>
v22.31 trial (next.html only): audit QT-12 — Vendors rows editable, a supplier name already on the list is updated instead of added twice
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T49gnSNZq31rPRt1vHk4Rc
</commit_message>
<xml_diff>
--- a/nexidoc/Nexi_Purchasing_Audit_v22.31.xlsx
+++ b/nexidoc/Nexi_Purchasing_Audit_v22.31.xlsx
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7"/>
@@ -2316,12 +2316,16 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr"/>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Partly v22.31 (trial)</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Vendors rows can be edited; adding an existing name offers to update it (test purch-audit-v2231). The other writers still append by name.</t>
+        </is>
+      </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Three writers append vendors with no duplicate check; the Vendors list has no edit.</t>

</xml_diff>